<commit_message>
chore(data): actualizar consolidado automático [2026-08-05]
Ejecución automática del pipeline ETL.
Año cierre: 2026
Disparado por: schedule
Run ID: 30990351609
</commit_message>
<xml_diff>
--- a/data/raw/Fuentes Consolidadas/Indicadores Kawak.xlsx
+++ b/data/raw/Fuentes Consolidadas/Indicadores Kawak.xlsx
@@ -3539,8 +3539,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3556,7 +3564,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -3564,12 +3572,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3868,31 +3894,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): actualizar consolidado automático [2026-09-05]
Ejecución automática del pipeline ETL.
Año cierre: 2026
Disparado por: schedule
Run ID: 33960541292
</commit_message>
<xml_diff>
--- a/data/raw/Fuentes Consolidadas/Indicadores Kawak.xlsx
+++ b/data/raw/Fuentes Consolidadas/Indicadores Kawak.xlsx
@@ -3599,8 +3599,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -3616,7 +3624,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -3624,12 +3632,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3928,31 +3954,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>